<commit_message>
Add 3 more products: resource histogram, workforce plan, schedule risk starter kit
</commit_message>
<xml_diff>
--- a/products/3-Week Lookahead Starter Template.xlsx
+++ b/products/3-Week Lookahead Starter Template.xlsx
@@ -17,8 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="mmm d, yyyy"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -805,15 +806,11 @@
           <t>J. Smith</t>
         </is>
       </c>
-      <c r="E6" s="11" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
-      <c r="F6" s="11" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
+      <c r="E6" s="11" t="n">
+        <v>46237</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>46241</v>
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Professional polish pass: branded footers, doc properties, print setup, tab colors, PDF footer/rule
</commit_message>
<xml_diff>
--- a/products/3-Week Lookahead Starter Template.xlsx
+++ b/products/3-Week Lookahead Starter Template.xlsx
@@ -10,7 +10,9 @@
     <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="3-Week Lookahead" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'3-Week Lookahead'!$3:$4</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -21,7 +23,7 @@
     <numFmt numFmtId="164" formatCode="mmm d, yyyy"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -88,6 +90,12 @@
       <name val="Arial"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="0033415C"/>
+      <sz val="8"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -112,7 +120,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -134,11 +142,16 @@
         <color rgb="00DDE3EA"/>
       </bottom>
     </border>
+    <border>
+      <top style="thin">
+        <color rgb="00DDE3EA"/>
+      </top>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -178,6 +191,8 @@
     <xf numFmtId="0" fontId="11" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="11" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="11" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -540,6 +555,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="0014213D"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -626,10 +642,11 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="000F766E"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Q30"/>
+  <dimension ref="A1:Q32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1383,8 +1400,31 @@
       </c>
       <c r="Q30" s="16" t="n"/>
     </row>
+    <row r="32">
+      <c r="A32" s="19" t="inlineStr">
+        <is>
+          <t>CPM Toolkit  |  3-Week Lookahead Starter Template  |  v1.0</t>
+        </is>
+      </c>
+      <c r="B32" s="20" t="n"/>
+      <c r="C32" s="20" t="n"/>
+      <c r="D32" s="20" t="n"/>
+      <c r="E32" s="20" t="n"/>
+      <c r="F32" s="20" t="n"/>
+      <c r="G32" s="20" t="n"/>
+      <c r="H32" s="20" t="n"/>
+      <c r="I32" s="20" t="n"/>
+      <c r="J32" s="20" t="n"/>
+      <c r="K32" s="20" t="n"/>
+      <c r="L32" s="20" t="n"/>
+      <c r="M32" s="20" t="n"/>
+      <c r="N32" s="20" t="n"/>
+      <c r="O32" s="20" t="n"/>
+      <c r="P32" s="20" t="n"/>
+      <c r="Q32" s="20" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="16">
     <mergeCell ref="C3:C4"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="A3:A4"/>
@@ -1399,8 +1439,11 @@
     <mergeCell ref="O3:O4"/>
     <mergeCell ref="Q3:Q4"/>
     <mergeCell ref="P3:P4"/>
+    <mergeCell ref="A32:Q32"/>
     <mergeCell ref="A5:Q5"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.35" right="0.35" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix 2 formula bugs found by live-Excel testing: guarded AVERAGE/MAX and Days Remaining on blank rows. Add repeatable Excel COM error-scan test.
</commit_message>
<xml_diff>
--- a/products/3-Week Lookahead Starter Template.xlsx
+++ b/products/3-Week Lookahead Starter Template.xlsx
@@ -863,7 +863,7 @@
         </is>
       </c>
       <c r="P6" s="12">
-        <f>F6-TODAY()</f>
+        <f>IF(F6&lt;&gt;"",F6-TODAY(),"")</f>
         <v/>
       </c>
       <c r="Q6" s="10" t="inlineStr">
@@ -889,7 +889,7 @@
       <c r="N7" s="13" t="n"/>
       <c r="O7" s="13" t="n"/>
       <c r="P7" s="15">
-        <f>F7-TODAY()</f>
+        <f>IF(F7&lt;&gt;"",F7-TODAY(),"")</f>
         <v/>
       </c>
       <c r="Q7" s="13" t="n"/>
@@ -911,7 +911,7 @@
       <c r="N8" s="16" t="n"/>
       <c r="O8" s="16" t="n"/>
       <c r="P8" s="18">
-        <f>F8-TODAY()</f>
+        <f>IF(F8&lt;&gt;"",F8-TODAY(),"")</f>
         <v/>
       </c>
       <c r="Q8" s="16" t="n"/>
@@ -933,7 +933,7 @@
       <c r="N9" s="13" t="n"/>
       <c r="O9" s="13" t="n"/>
       <c r="P9" s="15">
-        <f>F9-TODAY()</f>
+        <f>IF(F9&lt;&gt;"",F9-TODAY(),"")</f>
         <v/>
       </c>
       <c r="Q9" s="13" t="n"/>
@@ -955,7 +955,7 @@
       <c r="N10" s="16" t="n"/>
       <c r="O10" s="16" t="n"/>
       <c r="P10" s="18">
-        <f>F10-TODAY()</f>
+        <f>IF(F10&lt;&gt;"",F10-TODAY(),"")</f>
         <v/>
       </c>
       <c r="Q10" s="16" t="n"/>
@@ -977,7 +977,7 @@
       <c r="N11" s="13" t="n"/>
       <c r="O11" s="13" t="n"/>
       <c r="P11" s="15">
-        <f>F11-TODAY()</f>
+        <f>IF(F11&lt;&gt;"",F11-TODAY(),"")</f>
         <v/>
       </c>
       <c r="Q11" s="13" t="n"/>
@@ -999,7 +999,7 @@
       <c r="N12" s="16" t="n"/>
       <c r="O12" s="16" t="n"/>
       <c r="P12" s="18">
-        <f>F12-TODAY()</f>
+        <f>IF(F12&lt;&gt;"",F12-TODAY(),"")</f>
         <v/>
       </c>
       <c r="Q12" s="16" t="n"/>
@@ -1021,7 +1021,7 @@
       <c r="N13" s="13" t="n"/>
       <c r="O13" s="13" t="n"/>
       <c r="P13" s="15">
-        <f>F13-TODAY()</f>
+        <f>IF(F13&lt;&gt;"",F13-TODAY(),"")</f>
         <v/>
       </c>
       <c r="Q13" s="13" t="n"/>
@@ -1043,7 +1043,7 @@
       <c r="N14" s="16" t="n"/>
       <c r="O14" s="16" t="n"/>
       <c r="P14" s="18">
-        <f>F14-TODAY()</f>
+        <f>IF(F14&lt;&gt;"",F14-TODAY(),"")</f>
         <v/>
       </c>
       <c r="Q14" s="16" t="n"/>
@@ -1065,7 +1065,7 @@
       <c r="N15" s="13" t="n"/>
       <c r="O15" s="13" t="n"/>
       <c r="P15" s="15">
-        <f>F15-TODAY()</f>
+        <f>IF(F15&lt;&gt;"",F15-TODAY(),"")</f>
         <v/>
       </c>
       <c r="Q15" s="13" t="n"/>
@@ -1087,7 +1087,7 @@
       <c r="N16" s="16" t="n"/>
       <c r="O16" s="16" t="n"/>
       <c r="P16" s="18">
-        <f>F16-TODAY()</f>
+        <f>IF(F16&lt;&gt;"",F16-TODAY(),"")</f>
         <v/>
       </c>
       <c r="Q16" s="16" t="n"/>
@@ -1109,7 +1109,7 @@
       <c r="N17" s="13" t="n"/>
       <c r="O17" s="13" t="n"/>
       <c r="P17" s="15">
-        <f>F17-TODAY()</f>
+        <f>IF(F17&lt;&gt;"",F17-TODAY(),"")</f>
         <v/>
       </c>
       <c r="Q17" s="13" t="n"/>
@@ -1131,7 +1131,7 @@
       <c r="N18" s="16" t="n"/>
       <c r="O18" s="16" t="n"/>
       <c r="P18" s="18">
-        <f>F18-TODAY()</f>
+        <f>IF(F18&lt;&gt;"",F18-TODAY(),"")</f>
         <v/>
       </c>
       <c r="Q18" s="16" t="n"/>
@@ -1153,7 +1153,7 @@
       <c r="N19" s="13" t="n"/>
       <c r="O19" s="13" t="n"/>
       <c r="P19" s="15">
-        <f>F19-TODAY()</f>
+        <f>IF(F19&lt;&gt;"",F19-TODAY(),"")</f>
         <v/>
       </c>
       <c r="Q19" s="13" t="n"/>
@@ -1175,7 +1175,7 @@
       <c r="N20" s="16" t="n"/>
       <c r="O20" s="16" t="n"/>
       <c r="P20" s="18">
-        <f>F20-TODAY()</f>
+        <f>IF(F20&lt;&gt;"",F20-TODAY(),"")</f>
         <v/>
       </c>
       <c r="Q20" s="16" t="n"/>
@@ -1197,7 +1197,7 @@
       <c r="N21" s="13" t="n"/>
       <c r="O21" s="13" t="n"/>
       <c r="P21" s="15">
-        <f>F21-TODAY()</f>
+        <f>IF(F21&lt;&gt;"",F21-TODAY(),"")</f>
         <v/>
       </c>
       <c r="Q21" s="13" t="n"/>
@@ -1219,7 +1219,7 @@
       <c r="N22" s="16" t="n"/>
       <c r="O22" s="16" t="n"/>
       <c r="P22" s="18">
-        <f>F22-TODAY()</f>
+        <f>IF(F22&lt;&gt;"",F22-TODAY(),"")</f>
         <v/>
       </c>
       <c r="Q22" s="16" t="n"/>
@@ -1241,7 +1241,7 @@
       <c r="N23" s="13" t="n"/>
       <c r="O23" s="13" t="n"/>
       <c r="P23" s="15">
-        <f>F23-TODAY()</f>
+        <f>IF(F23&lt;&gt;"",F23-TODAY(),"")</f>
         <v/>
       </c>
       <c r="Q23" s="13" t="n"/>
@@ -1263,7 +1263,7 @@
       <c r="N24" s="16" t="n"/>
       <c r="O24" s="16" t="n"/>
       <c r="P24" s="18">
-        <f>F24-TODAY()</f>
+        <f>IF(F24&lt;&gt;"",F24-TODAY(),"")</f>
         <v/>
       </c>
       <c r="Q24" s="16" t="n"/>
@@ -1285,7 +1285,7 @@
       <c r="N25" s="13" t="n"/>
       <c r="O25" s="13" t="n"/>
       <c r="P25" s="15">
-        <f>F25-TODAY()</f>
+        <f>IF(F25&lt;&gt;"",F25-TODAY(),"")</f>
         <v/>
       </c>
       <c r="Q25" s="13" t="n"/>
@@ -1307,7 +1307,7 @@
       <c r="N26" s="16" t="n"/>
       <c r="O26" s="16" t="n"/>
       <c r="P26" s="18">
-        <f>F26-TODAY()</f>
+        <f>IF(F26&lt;&gt;"",F26-TODAY(),"")</f>
         <v/>
       </c>
       <c r="Q26" s="16" t="n"/>
@@ -1329,7 +1329,7 @@
       <c r="N27" s="13" t="n"/>
       <c r="O27" s="13" t="n"/>
       <c r="P27" s="15">
-        <f>F27-TODAY()</f>
+        <f>IF(F27&lt;&gt;"",F27-TODAY(),"")</f>
         <v/>
       </c>
       <c r="Q27" s="13" t="n"/>
@@ -1351,7 +1351,7 @@
       <c r="N28" s="16" t="n"/>
       <c r="O28" s="16" t="n"/>
       <c r="P28" s="18">
-        <f>F28-TODAY()</f>
+        <f>IF(F28&lt;&gt;"",F28-TODAY(),"")</f>
         <v/>
       </c>
       <c r="Q28" s="16" t="n"/>
@@ -1373,7 +1373,7 @@
       <c r="N29" s="13" t="n"/>
       <c r="O29" s="13" t="n"/>
       <c r="P29" s="15">
-        <f>F29-TODAY()</f>
+        <f>IF(F29&lt;&gt;"",F29-TODAY(),"")</f>
         <v/>
       </c>
       <c r="Q29" s="13" t="n"/>
@@ -1395,7 +1395,7 @@
       <c r="N30" s="16" t="n"/>
       <c r="O30" s="16" t="n"/>
       <c r="P30" s="18">
-        <f>F30-TODAY()</f>
+        <f>IF(F30&lt;&gt;"",F30-TODAY(),"")</f>
         <v/>
       </c>
       <c r="Q30" s="16" t="n"/>

</xml_diff>